<commit_message>
new ui, key shortcuts
</commit_message>
<xml_diff>
--- a/dist/time_tracker_2026-04-10.xlsx
+++ b/dist/time_tracker_2026-04-10.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1956,49 +1956,41 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-04-10T12:12:45.295784</t>
+          <t>2026-04-10T12:07:10.994000</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-04-10T12:12:54.761578</t>
+          <t>2026-04-10T15:07:10.995000</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>DEUTZ-DE-21-01-00</t>
+          <t>Black-Jack</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>S-2102386707</t>
+          <t>104180001560</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>114012</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>0130</t>
-        </is>
-      </c>
+          <t>114000</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>D330000</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>!"§$%&amp;/()=?ß´`,.-;:_öäü'#+*~&lt;&gt;|^°aâa</t>
-        </is>
-      </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -2006,12 +1998,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-04-10T12:32:21.341568</t>
+          <t>2026-04-10T12:12:45.295784</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-04-10T12:32:33.653295</t>
+          <t>2026-04-10T12:12:54.761578</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2021,17 +2013,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>HYUN-DE-25-07-00</t>
+          <t>DEUTZ-DE-21-01-00</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>S-2104168132</t>
+          <t>S-2102386707</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>114000</t>
+          <t>114012</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2046,7 +2038,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>test 07</t>
+          <t>!"§$%&amp;/()=?ß´`,.-;:_öäü'#+*~&lt;&gt;|^°aâa</t>
         </is>
       </c>
     </row>
@@ -2056,12 +2048,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-04-10T13:35:45.540126</t>
+          <t>2026-04-10T12:32:21.341568</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-04-10T13:35:49.084112</t>
+          <t>2026-04-10T12:32:33.653295</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2094,7 +2086,11 @@
           <t>D330000</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>test 07</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -2102,12 +2098,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-04-10T13:42:03.614955</t>
+          <t>2026-04-10T13:35:45.540126</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-04-10T13:42:14.255434</t>
+          <t>2026-04-10T13:35:49.084112</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2117,12 +2113,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Black-Jack</t>
+          <t>HYUN-DE-25-07-00</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>104180001560</t>
+          <t>S-2104168132</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2130,17 +2126,17 @@
           <t>114000</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>0130</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>D330000</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>test if comment is working after starting</t>
-        </is>
-      </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2148,12 +2144,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-04-10T13:42:19.346547</t>
+          <t>2026-04-10T13:42:03.614955</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-04-10T13:42:22.367727</t>
+          <t>2026-04-10T13:42:14.255434</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2163,12 +2159,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>HYUN-DE-25-07-00</t>
+          <t>Black-Jack</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>S-2104168132</t>
+          <t>104180001560</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2176,11 +2172,7 @@
           <t>114000</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>0130</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>D330000</t>
@@ -2188,7 +2180,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>test 07</t>
+          <t>test if comment is working after starting</t>
         </is>
       </c>
     </row>
@@ -2198,12 +2190,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-04-10T14:04:58.126959</t>
+          <t>2026-04-10T13:42:19.346547</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-04-10T14:05:02.279455</t>
+          <t>2026-04-10T13:42:22.367727</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2213,12 +2205,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Black-Jack</t>
+          <t>HYUN-DE-25-07-00</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>104180001560</t>
+          <t>S-2104168132</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2226,7 +2218,11 @@
           <t>114000</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>0130</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>D330000</t>
@@ -2234,7 +2230,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>test entry table 05</t>
+          <t>test 07</t>
         </is>
       </c>
     </row>
@@ -2244,12 +2240,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-04-10T14:26:13.873224</t>
+          <t>2026-04-10T14:04:58.126959</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-04-10T14:26:19.152946</t>
+          <t>2026-04-10T14:05:02.279455</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2259,12 +2255,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Gemeinkosten</t>
+          <t>Black-Jack</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>8001233873</t>
+          <t>104180001560</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2272,17 +2268,17 @@
           <t>114000</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>0130</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>D330000</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>test entry table 05</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -2290,45 +2286,137 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>2026-04-10T14:26:13.873224</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-04-10T14:26:19.152946</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Gemeinkosten</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>8001233873</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>114000</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>0130</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>D330000</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-04-10T14:52:20.362246</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-04-10T14:52:27.123069</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Black-Jack</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>104180001560</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>114000</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>D330000</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>ttt</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>2026-04-10T13:49:41</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>2026-04-10T13:49:44</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>HYUN-DE-25-07-00</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>S-2104168132</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>114000</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>0130</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>0130</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>D330020</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>test entry tableeeeee</t>
         </is>
@@ -2367,7 +2455,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15.04</v>
+        <v>18.04</v>
       </c>
     </row>
     <row r="3">
@@ -2377,7 +2465,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4">
@@ -2388,7 +2476,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-04-10 14:26:34</t>
+          <t>2026-04-10 15:07:37</t>
         </is>
       </c>
     </row>

</xml_diff>